<commit_message>
44 - Updated documentation
</commit_message>
<xml_diff>
--- a/documentation/TimeTracking.xlsx
+++ b/documentation/TimeTracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SWEN3Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B0353F-5E52-4394-B46D-A6F2C179199E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84B48F2-BD56-47B1-853B-0ECDA3D69A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="64">
   <si>
     <t>Team Member</t>
   </si>
@@ -201,6 +201,33 @@
   </si>
   <si>
     <t>Add integration tests</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>#39</t>
+  </si>
+  <si>
+    <t>Add MinIO service</t>
+  </si>
+  <si>
+    <t>#40</t>
+  </si>
+  <si>
+    <t>Integrate MinIO into REST server</t>
+  </si>
+  <si>
+    <t>#41</t>
+  </si>
+  <si>
+    <t>Integrate MinIO into OCRWorker</t>
+  </si>
+  <si>
+    <t>#42</t>
+  </si>
+  <si>
+    <t>Install Tesseract + Ghostscript in OCR worker container</t>
   </si>
 </sst>
 </file>
@@ -341,9 +368,86 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right/>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <vertical style="thin">
+          <color auto="1"/>
+        </vertical>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
           <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
         </bottom>
       </border>
     </dxf>
@@ -372,83 +476,6 @@
         </vertical>
       </border>
     </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right/>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <vertical style="thin">
-          <color auto="1"/>
-        </vertical>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -463,14 +490,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E23" totalsRowShown="0" headerRowDxfId="1" headerRowBorderDxfId="0" tableBorderDxfId="7" headerRowCellStyle="Heading 3">
-  <autoFilter ref="A1:E23" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E27" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" headerRowCellStyle="Heading 3">
+  <autoFilter ref="A1:E27" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{6A66199F-352C-41CA-BBFF-93091D04DBF3}" name="Sprint" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{150DA361-AB43-483E-A895-C2B5AEFE5F17}" name="Task ID" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{E63035FE-C75C-47CA-9048-6D3E90F64B6E}" name="Task Name" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{64F3594D-D4DA-4C6A-9302-5982481D8956}" name="Team Member" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{B25F98ED-A27D-43B2-83DE-4E79C37F47D1}" name="Time Invested (h)" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{6A66199F-352C-41CA-BBFF-93091D04DBF3}" name="Sprint" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{150DA361-AB43-483E-A895-C2B5AEFE5F17}" name="Task ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{E63035FE-C75C-47CA-9048-6D3E90F64B6E}" name="Task Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{64F3594D-D4DA-4C6A-9302-5982481D8956}" name="Team Member" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{B25F98ED-A27D-43B2-83DE-4E79C37F47D1}" name="Time Invested (h)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -739,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
@@ -1141,6 +1168,74 @@
         <v>2</v>
       </c>
     </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="3">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
55 - Updated Documentation
</commit_message>
<xml_diff>
--- a/documentation/TimeTracking.xlsx
+++ b/documentation/TimeTracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SWEN3Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44CC9D0A-8759-49D9-95AC-B3574C0CB5BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBED33C2-975F-42C9-83DE-787682795C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="79">
   <si>
     <t>Team Member</t>
   </si>
@@ -240,6 +240,39 @@
   </si>
   <si>
     <t>Add IOcrEngine abstraction and TesseractOcrEngine implementation</t>
+  </si>
+  <si>
+    <t>Sprint 5</t>
+  </si>
+  <si>
+    <t>#51</t>
+  </si>
+  <si>
+    <t>Extend docker-compose for Gemini</t>
+  </si>
+  <si>
+    <t>#52</t>
+  </si>
+  <si>
+    <t>Set up GenAiWorker</t>
+  </si>
+  <si>
+    <t>#53</t>
+  </si>
+  <si>
+    <t>Connect GenAiWorker to OcrWorker</t>
+  </si>
+  <si>
+    <t>#55</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>#28</t>
+  </si>
+  <si>
+    <t>Add Adminer for DB management</t>
   </si>
 </sst>
 </file>
@@ -441,25 +474,25 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
+      <border>
         <bottom style="thin">
-          <color auto="1"/>
+          <color theme="1"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
         <bottom style="thin">
-          <color theme="1"/>
+          <color auto="1"/>
         </bottom>
       </border>
     </dxf>
@@ -502,8 +535,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E29" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" headerRowCellStyle="Heading 3">
-  <autoFilter ref="A1:E29" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E34" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" headerRowCellStyle="Heading 3">
+  <autoFilter ref="A1:E34" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{6A66199F-352C-41CA-BBFF-93091D04DBF3}" name="Sprint" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{150DA361-AB43-483E-A895-C2B5AEFE5F17}" name="Task ID" dataDxfId="3"/>
@@ -778,7 +811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
@@ -1282,6 +1315,91 @@
         <v>7</v>
       </c>
     </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="3">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="3">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="3">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
79 - Updated documentation
</commit_message>
<xml_diff>
--- a/documentation/TimeTracking.xlsx
+++ b/documentation/TimeTracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SWEN3Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBED33C2-975F-42C9-83DE-787682795C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F7197D-468B-44CE-B2AD-94FF966E3FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="104">
   <si>
     <t>Team Member</t>
   </si>
@@ -273,6 +273,81 @@
   </si>
   <si>
     <t>Add Adminer for DB management</t>
+  </si>
+  <si>
+    <t>Sprint 6</t>
+  </si>
+  <si>
+    <t>#67</t>
+  </si>
+  <si>
+    <t>Documentation for Sprint 6</t>
+  </si>
+  <si>
+    <t>#60</t>
+  </si>
+  <si>
+    <t>Add ElasticSearch to docker-compose</t>
+  </si>
+  <si>
+    <t>#61</t>
+  </si>
+  <si>
+    <t>ElasticSearch Document Indexing by Rest Server</t>
+  </si>
+  <si>
+    <t>#63</t>
+  </si>
+  <si>
+    <t>ElasticSearch Document Search by Rest Server</t>
+  </si>
+  <si>
+    <t>#66</t>
+  </si>
+  <si>
+    <t>#62</t>
+  </si>
+  <si>
+    <t>Search in Frontend</t>
+  </si>
+  <si>
+    <t>#64</t>
+  </si>
+  <si>
+    <t>Unit Tests for ElasticSearch in REST server</t>
+  </si>
+  <si>
+    <t>Develop an additional use case</t>
+  </si>
+  <si>
+    <t>#68</t>
+  </si>
+  <si>
+    <t>Implement Use Case in REST server</t>
+  </si>
+  <si>
+    <t>#69</t>
+  </si>
+  <si>
+    <t>Implement Use Case in Frontend</t>
+  </si>
+  <si>
+    <t>#71</t>
+  </si>
+  <si>
+    <t>Elastic Search Documentation</t>
+  </si>
+  <si>
+    <t>#73</t>
+  </si>
+  <si>
+    <t>Documentation for Use Case</t>
+  </si>
+  <si>
+    <t>#79</t>
+  </si>
+  <si>
+    <t>Finalized Documentation</t>
   </si>
 </sst>
 </file>
@@ -535,8 +610,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E34" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" headerRowCellStyle="Heading 3">
-  <autoFilter ref="A1:E34" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E46" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" headerRowCellStyle="Heading 3">
+  <autoFilter ref="A1:E46" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{6A66199F-352C-41CA-BBFF-93091D04DBF3}" name="Sprint" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{150DA361-AB43-483E-A895-C2B5AEFE5F17}" name="Task ID" dataDxfId="3"/>
@@ -811,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
@@ -1400,6 +1475,210 @@
         <v>1</v>
       </c>
     </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E40" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="3">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
90 - Updated documentation
</commit_message>
<xml_diff>
--- a/documentation/TimeTracking.xlsx
+++ b/documentation/TimeTracking.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\SWEN3Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F7197D-468B-44CE-B2AD-94FF966E3FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2790B893-1560-4090-9CC7-5A4FC03EE7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="112">
   <si>
     <t>Team Member</t>
   </si>
@@ -348,6 +348,30 @@
   </si>
   <si>
     <t>Finalized Documentation</t>
+  </si>
+  <si>
+    <t>Sprint 7</t>
+  </si>
+  <si>
+    <t>#84</t>
+  </si>
+  <si>
+    <t>Health Checks in Docker-Compose</t>
+  </si>
+  <si>
+    <t>#85</t>
+  </si>
+  <si>
+    <t>Batch Processor</t>
+  </si>
+  <si>
+    <t>#86</t>
+  </si>
+  <si>
+    <t>Finalize Integration Test</t>
+  </si>
+  <si>
+    <t>#90</t>
   </si>
 </sst>
 </file>
@@ -610,8 +634,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E46" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" headerRowCellStyle="Heading 3">
-  <autoFilter ref="A1:E46" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}" name="Table1" displayName="Table1" ref="A1:E50" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" headerRowCellStyle="Heading 3">
+  <autoFilter ref="A1:E50" xr:uid="{84928939-512D-4669-9CEB-C940ECF23420}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{6A66199F-352C-41CA-BBFF-93091D04DBF3}" name="Sprint" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{150DA361-AB43-483E-A895-C2B5AEFE5F17}" name="Task ID" dataDxfId="3"/>
@@ -886,7 +910,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
@@ -1679,6 +1703,74 @@
         <v>1</v>
       </c>
     </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E50" s="3">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>